<commit_message>
Place demonstration experiment 29 in row 30 and remove unused fields
</commit_message>
<xml_diff>
--- a/sample_data/atomization_summary_template.xlsx
+++ b/sample_data/atomization_summary_template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测量数据" sheetId="1" r:id="R2fa3efcb16654624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测量数据" sheetId="1" r:id="R08d7c4c094be4675"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -198,7 +198,7 @@
     <x:xf numFmtId="200" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -411,7 +411,7 @@
     <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="32" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
@@ -426,13 +426,13 @@
     <x:col min="21" max="21" width="12" hidden="0" customWidth="1"/>
     <x:col min="22" max="22" width="12" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="12" hidden="0" customWidth="1"/>
-    <x:col min="24" max="24" width="12" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="13" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="13" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="12" hidden="0" customWidth="1"/>
     <x:col min="26" max="26" width="12" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="12" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="12" hidden="0" customWidth="1"/>
-    <x:col min="29" max="29" width="12" hidden="0" customWidth="1"/>
-    <x:col min="30" max="30" width="44" hidden="0" customWidth="1"/>
+    <x:col min="29" max="29" width="44" hidden="0" customWidth="1"/>
+    <x:col min="30" max="30" width="12" hidden="0" customWidth="1"/>
     <x:col min="31" max="31" width="12" hidden="0" customWidth="1"/>
     <x:col min="32" max="32" width="12" hidden="0" customWidth="1"/>
     <x:col min="33" max="33" width="12" hidden="0" customWidth="1"/>
@@ -440,16 +440,16 @@
     <x:col min="35" max="35" width="12" hidden="0" customWidth="1"/>
     <x:col min="36" max="36" width="12" hidden="0" customWidth="1"/>
     <x:col min="37" max="37" width="12" hidden="0" customWidth="1"/>
-    <x:col min="38" max="38" width="12" hidden="0" customWidth="1"/>
-    <x:col min="39" max="39" width="20" hidden="0" customWidth="1"/>
+    <x:col min="38" max="38" width="20" hidden="0" customWidth="1"/>
+    <x:col min="39" max="39" width="12" hidden="0" customWidth="1"/>
     <x:col min="40" max="40" width="12" hidden="0" customWidth="1"/>
     <x:col min="41" max="41" width="12" hidden="0" customWidth="1"/>
     <x:col min="42" max="42" width="12" hidden="0" customWidth="1"/>
     <x:col min="43" max="43" width="12" hidden="0" customWidth="1"/>
     <x:col min="44" max="44" width="12" hidden="0" customWidth="1"/>
     <x:col min="45" max="45" width="12" hidden="0" customWidth="1"/>
-    <x:col min="46" max="46" width="12" hidden="0" customWidth="1"/>
-    <x:col min="47" max="47" width="20" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="20" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="12" hidden="0" customWidth="1"/>
     <x:col min="48" max="48" width="12" hidden="0" customWidth="1"/>
     <x:col min="49" max="49" width="12" hidden="0" customWidth="1"/>
     <x:col min="50" max="50" width="12" hidden="0" customWidth="1"/>
@@ -458,11 +458,10 @@
     <x:col min="53" max="53" width="12" hidden="0" customWidth="1"/>
     <x:col min="54" max="54" width="12" hidden="0" customWidth="1"/>
     <x:col min="55" max="55" width="12" hidden="0" customWidth="1"/>
-    <x:col min="56" max="56" width="12" hidden="0" customWidth="1"/>
-    <x:col min="57" max="57" width="20" hidden="0" customWidth="1"/>
+    <x:col min="56" max="56" width="20" hidden="0" customWidth="1"/>
+    <x:col min="57" max="57" width="12" hidden="0" customWidth="1"/>
     <x:col min="58" max="58" width="12" hidden="0" customWidth="1"/>
-    <x:col min="59" max="59" width="12" hidden="0" customWidth="1"/>
-    <x:col min="60" max="60" width="20" hidden="0" customWidth="1"/>
+    <x:col min="59" max="59" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -490,171 +489,163 @@
       <x:c r="H1" s="28" t="str">
         <x:v>ExpIntEndFrame</x:v>
       </x:c>
-      <x:c r="I1" s="28" t="str">
-        <x:v>图像备注</x:v>
-      </x:c>
-      <x:c r="J1" s="29" t="str">
+      <x:c r="I1" s="29" t="str">
         <x:v>U</x:v>
       </x:c>
-      <x:c r="K1" s="27" t="str">
+      <x:c r="J1" s="27" t="str">
         <x:v>DU</x:v>
       </x:c>
-      <x:c r="L1" s="29" t="str">
+      <x:c r="K1" s="29" t="str">
         <x:v>Pc</x:v>
       </x:c>
-      <x:c r="M1" s="27" t="str">
+      <x:c r="L1" s="27" t="str">
         <x:v>DPc</x:v>
       </x:c>
+      <x:c r="M1" s="28" t="str">
+        <x:v>CdIntStart</x:v>
+      </x:c>
       <x:c r="N1" s="28" t="str">
-        <x:v>CdIntStart</x:v>
-      </x:c>
-      <x:c r="O1" s="28" t="str">
         <x:v>CdIntEnd</x:v>
       </x:c>
-      <x:c r="P1" s="30" t="str">
+      <x:c r="O1" s="30" t="str">
         <x:v>cd</x:v>
       </x:c>
-      <x:c r="Q1" s="27" t="str">
+      <x:c r="P1" s="27" t="str">
         <x:v>Dcd</x:v>
       </x:c>
-      <x:c r="R1" s="30" t="str">
+      <x:c r="Q1" s="30" t="str">
         <x:v>Pccd</x:v>
       </x:c>
-      <x:c r="S1" s="27" t="str">
+      <x:c r="R1" s="27" t="str">
         <x:v>DPccd</x:v>
       </x:c>
-      <x:c r="T1" s="30" t="str">
+      <x:c r="S1" s="30" t="str">
         <x:v>DPcd</x:v>
       </x:c>
+      <x:c r="T1" s="27" t="str">
+        <x:v>DDPcd</x:v>
+      </x:c>
       <x:c r="U1" s="27" t="str">
-        <x:v>DDPcd</x:v>
+        <x:v>真实DP</x:v>
       </x:c>
       <x:c r="V1" s="27" t="str">
-        <x:v>真实DP</x:v>
+        <x:v>真实K</x:v>
       </x:c>
       <x:c r="W1" s="27" t="str">
-        <x:v>真实K</x:v>
+        <x:v>K</x:v>
       </x:c>
       <x:c r="X1" s="27" t="str">
-        <x:v>K</x:v>
+        <x:v>Q2</x:v>
       </x:c>
       <x:c r="Y1" s="27" t="str">
-        <x:v>Q2</x:v>
+        <x:v>Q2*</x:v>
       </x:c>
       <x:c r="Z1" s="27" t="str">
-        <x:v>Q2*</x:v>
+        <x:v>cd*</x:v>
       </x:c>
       <x:c r="AA1" s="27" t="str">
-        <x:v>cd*</x:v>
+        <x:v>U*</x:v>
       </x:c>
       <x:c r="AB1" s="27" t="str">
-        <x:v>U*</x:v>
+        <x:v>图像问题</x:v>
       </x:c>
       <x:c r="AC1" s="27" t="str">
-        <x:v>图像问题</x:v>
+        <x:v>备注</x:v>
       </x:c>
       <x:c r="AD1" s="27" t="str">
-        <x:v>备注</x:v>
+        <x:v>代表图</x:v>
       </x:c>
       <x:c r="AE1" s="27" t="str">
-        <x:v>代表图</x:v>
-      </x:c>
-      <x:c r="AF1" s="27" t="str">
         <x:v>模式</x:v>
       </x:c>
+      <x:c r="AF1" s="31" t="str">
+        <x:v>XLeft</x:v>
+      </x:c>
       <x:c r="AG1" s="31" t="str">
-        <x:v>XLeft</x:v>
+        <x:v>XRight</x:v>
       </x:c>
       <x:c r="AH1" s="31" t="str">
-        <x:v>XRight</x:v>
+        <x:v>Y</x:v>
       </x:c>
       <x:c r="AI1" s="31" t="str">
-        <x:v>Y</x:v>
+        <x:v>Rmax</x:v>
       </x:c>
       <x:c r="AJ1" s="31" t="str">
-        <x:v>Rmax</x:v>
+        <x:v>ThetaLeft</x:v>
       </x:c>
       <x:c r="AK1" s="31" t="str">
-        <x:v>ThetaLeft</x:v>
+        <x:v>ThetaRight</x:v>
       </x:c>
       <x:c r="AL1" s="31" t="str">
-        <x:v>ThetaRight</x:v>
+        <x:v>window_length</x:v>
       </x:c>
       <x:c r="AM1" s="31" t="str">
-        <x:v>window_length</x:v>
+        <x:v>polyorder</x:v>
       </x:c>
       <x:c r="AN1" s="31" t="str">
-        <x:v>polyorder</x:v>
+        <x:v>NumAvgL</x:v>
       </x:c>
       <x:c r="AO1" s="31" t="str">
-        <x:v>NumAvgL</x:v>
+        <x:v>RStartL</x:v>
       </x:c>
       <x:c r="AP1" s="31" t="str">
-        <x:v>RStartL</x:v>
+        <x:v>NumAvgR</x:v>
       </x:c>
       <x:c r="AQ1" s="31" t="str">
-        <x:v>NumAvgR</x:v>
+        <x:v>RStartR</x:v>
       </x:c>
       <x:c r="AR1" s="31" t="str">
-        <x:v>RStartR</x:v>
+        <x:v>ThresRatioL</x:v>
       </x:c>
       <x:c r="AS1" s="31" t="str">
-        <x:v>ThresRatioL</x:v>
+        <x:v>ThresRatioR</x:v>
       </x:c>
       <x:c r="AT1" s="31" t="str">
-        <x:v>ThresRatioR</x:v>
+        <x:v>num_processes</x:v>
       </x:c>
       <x:c r="AU1" s="31" t="str">
-        <x:v>num_processes</x:v>
-      </x:c>
-      <x:c r="AV1" s="31" t="str">
         <x:v>compute_time</x:v>
       </x:c>
-      <x:c r="AW1" s="32" t="str">
+      <x:c r="AV1" s="32" t="str">
         <x:v>AngleL</x:v>
       </x:c>
-      <x:c r="AX1" s="27" t="str">
+      <x:c r="AW1" s="27" t="str">
         <x:v>AngleLStd</x:v>
       </x:c>
-      <x:c r="AY1" s="33" t="str">
+      <x:c r="AX1" s="33" t="str">
         <x:v>AngleLRevStd</x:v>
       </x:c>
-      <x:c r="AZ1" s="32" t="str">
+      <x:c r="AY1" s="32" t="str">
         <x:v>AngleR</x:v>
       </x:c>
-      <x:c r="BA1" s="27" t="str">
+      <x:c r="AZ1" s="27" t="str">
         <x:v>AngleRStd</x:v>
       </x:c>
-      <x:c r="BB1" s="33" t="str">
+      <x:c r="BA1" s="33" t="str">
         <x:v>AngleRRevStd</x:v>
       </x:c>
-      <x:c r="BC1" s="32" t="str">
+      <x:c r="BB1" s="32" t="str">
         <x:v>AtmAngle</x:v>
       </x:c>
-      <x:c r="BD1" s="27" t="str">
+      <x:c r="BC1" s="27" t="str">
         <x:v>AtmAngleStd</x:v>
       </x:c>
-      <x:c r="BE1" s="33" t="str">
+      <x:c r="BD1" s="33" t="str">
         <x:v>AtmAngleRevStd</x:v>
       </x:c>
-      <x:c r="BF1" s="34" t="str">
+      <x:c r="BE1" s="34" t="str">
         <x:v>AngleM</x:v>
       </x:c>
+      <x:c r="BF1" s="33" t="str">
+        <x:v>AngleMStd</x:v>
+      </x:c>
       <x:c r="BG1" s="33" t="str">
-        <x:v>AngleMStd</x:v>
-      </x:c>
-      <x:c r="BH1" s="33" t="str">
         <x:v>AngleMRevStd</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="2" t="str">
-        <x:v>1pix</x:v>
-      </x:c>
-      <x:c r="B2" s="2" t="n">
-        <x:f>0.5/18</x:f>
-        <x:v>0.027777777777777776</x:v>
-      </x:c>
+      <x:c r="A2" s="2"/>
+      <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
       <x:c r="D2" s="2"/>
       <x:c r="E2" s="6" t="str">
@@ -669,54 +660,54 @@
       <x:c r="H2" s="6" t="str">
         <x:v>帧</x:v>
       </x:c>
-      <x:c r="I2" s="28"/>
-      <x:c r="J2" s="12" t="str">
+      <x:c r="I2" s="12" t="str">
         <x:v>m/s</x:v>
       </x:c>
-      <x:c r="K2" s="2" t="str">
+      <x:c r="J2" s="2" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="L2" s="12" t="str">
+      <x:c r="K2" s="12" t="str">
         <x:v>MPa</x:v>
       </x:c>
-      <x:c r="M2" s="2" t="str">
+      <x:c r="L2" s="2" t="str">
         <x:v>%</x:v>
+      </x:c>
+      <x:c r="M2" s="6" t="str">
+        <x:v>ms</x:v>
       </x:c>
       <x:c r="N2" s="6" t="str">
         <x:v>ms</x:v>
       </x:c>
-      <x:c r="O2" s="6" t="str">
-        <x:v>ms</x:v>
-      </x:c>
-      <x:c r="P2" s="16" t="n">
+      <x:c r="O2" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q2" s="2" t="str">
+      <x:c r="P2" s="2" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="R2" s="16" t="str">
+      <x:c r="Q2" s="16" t="str">
         <x:v>MPa</x:v>
       </x:c>
-      <x:c r="S2" s="2" t="str">
+      <x:c r="R2" s="2" t="str">
         <x:v>%</x:v>
       </x:c>
-      <x:c r="T2" s="16" t="str">
+      <x:c r="S2" s="16" t="str">
         <x:v>MPa</x:v>
       </x:c>
-      <x:c r="U2" s="2" t="str">
+      <x:c r="T2" s="2" t="str">
         <x:v>%</x:v>
       </x:c>
+      <x:c r="U2" s="2"/>
       <x:c r="V2" s="2"/>
       <x:c r="W2" s="2"/>
-      <x:c r="X2" s="2"/>
-      <x:c r="Y2" s="2" t="n">
+      <x:c r="X2" s="2" t="n">
         <x:v>-0.18</x:v>
       </x:c>
+      <x:c r="Y2" s="2"/>
       <x:c r="Z2" s="2"/>
       <x:c r="AA2" s="2"/>
       <x:c r="AB2" s="2"/>
-      <x:c r="AC2" s="2"/>
-      <x:c r="AD2" s="27"/>
+      <x:c r="AC2" s="27"/>
+      <x:c r="AD2" s="2"/>
       <x:c r="AE2" s="2"/>
       <x:c r="AF2" s="2"/>
       <x:c r="AG2" s="2"/>
@@ -734,174 +725,251 @@
       <x:c r="AS2" s="2"/>
       <x:c r="AT2" s="2"/>
       <x:c r="AU2" s="2"/>
-      <x:c r="AV2" s="2"/>
-      <x:c r="AW2" s="21"/>
-      <x:c r="AX2" s="2"/>
-      <x:c r="AY2" s="24"/>
-      <x:c r="AZ2" s="21"/>
-      <x:c r="BA2" s="2"/>
-      <x:c r="BB2" s="24"/>
-      <x:c r="BC2" s="21"/>
-      <x:c r="BD2" s="2"/>
-      <x:c r="BE2" s="24"/>
-      <x:c r="BF2" s="26"/>
+      <x:c r="AV2" s="21"/>
+      <x:c r="AW2" s="2"/>
+      <x:c r="AX2" s="24"/>
+      <x:c r="AY2" s="21"/>
+      <x:c r="AZ2" s="2"/>
+      <x:c r="BA2" s="24"/>
+      <x:c r="BB2" s="21"/>
+      <x:c r="BC2" s="2"/>
+      <x:c r="BD2" s="24"/>
+      <x:c r="BE2" s="26"/>
+      <x:c r="BF2" s="24"/>
       <x:c r="BG2" s="24"/>
-      <x:c r="BH2" s="24"/>
-    </x:row>
-    <x:row r="3" ht="54" customHeight="1">
-      <x:c r="A3" s="2" t="n">
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="AC3" s="35"/>
+    </x:row>
+    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="AC4" s="35"/>
+    </x:row>
+    <x:row r="5" ht="28" customHeight="1">
+      <x:c r="AC5" s="35"/>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="AC6" s="35"/>
+    </x:row>
+    <x:row r="7" ht="28" customHeight="1">
+      <x:c r="AC7" s="35"/>
+    </x:row>
+    <x:row r="8" ht="28" customHeight="1">
+      <x:c r="AC8" s="35"/>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="AC9" s="35"/>
+    </x:row>
+    <x:row r="10" ht="28" customHeight="1">
+      <x:c r="AC10" s="35"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="AC11" s="35"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="AC12" s="35"/>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="AC13" s="35"/>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="AC14" s="35"/>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="AC15" s="35"/>
+    </x:row>
+    <x:row r="16" ht="28" customHeight="1">
+      <x:c r="AC16" s="35"/>
+    </x:row>
+    <x:row r="17" ht="28" customHeight="1">
+      <x:c r="AC17" s="35"/>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="AC18" s="35"/>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="AC19" s="35"/>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="AC20" s="35"/>
+    </x:row>
+    <x:row r="21" ht="28" customHeight="1">
+      <x:c r="AC21" s="35"/>
+    </x:row>
+    <x:row r="22" ht="28" customHeight="1">
+      <x:c r="AC22" s="35"/>
+    </x:row>
+    <x:row r="23" ht="28" customHeight="1">
+      <x:c r="AC23" s="35"/>
+    </x:row>
+    <x:row r="24" ht="28" customHeight="1">
+      <x:c r="AC24" s="35"/>
+    </x:row>
+    <x:row r="25" ht="28" customHeight="1">
+      <x:c r="AC25" s="35"/>
+    </x:row>
+    <x:row r="26" ht="28" customHeight="1">
+      <x:c r="AC26" s="35"/>
+    </x:row>
+    <x:row r="27" ht="28" customHeight="1">
+      <x:c r="AC27" s="35"/>
+    </x:row>
+    <x:row r="28" ht="28" customHeight="1">
+      <x:c r="AC28" s="35"/>
+    </x:row>
+    <x:row r="29" ht="28" customHeight="1">
+      <x:c r="AC29" s="35"/>
+    </x:row>
+    <x:row r="30" ht="54" customHeight="1">
+      <x:c r="A30" s="2" t="n">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="B3" s="4" t="str">
+      <x:c r="B30" s="4" t="str">
         <x:v>6-1-2</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="str">
+      <x:c r="C30" s="2" t="str">
         <x:v>C1MPa-3</x:v>
       </x:c>
-      <x:c r="D3" s="2"/>
-      <x:c r="E3" s="8" t="n">
+      <x:c r="D30" s="2"/>
+      <x:c r="E30" s="8" t="n">
         <x:v>525</x:v>
       </x:c>
-      <x:c r="F3" s="10" t="n">
-        <x:f>E3*40</x:f>
+      <x:c r="F30" s="10" t="n">
+        <x:f>E30*40</x:f>
         <x:v>21000</x:v>
       </x:c>
-      <x:c r="G3" s="8" t="n">
+      <x:c r="G30" s="8" t="n">
         <x:v>538</x:v>
       </x:c>
-      <x:c r="H3" s="10" t="n">
-        <x:f>G3*40</x:f>
+      <x:c r="H30" s="10" t="n">
+        <x:f>G30*40</x:f>
         <x:v>21520</x:v>
       </x:c>
-      <x:c r="I3" s="35" t="str">
-        <x:v>背景干扰太大，参数是特调的</x:v>
-      </x:c>
-      <x:c r="J3" s="13" t="n">
+      <x:c r="I30" s="13" t="n">
         <x:v>26.19499</x:v>
       </x:c>
-      <x:c r="K3" s="14" t="n">
+      <x:c r="J30" s="14" t="n">
         <x:v>1.71047</x:v>
       </x:c>
-      <x:c r="L3" s="13" t="n">
+      <x:c r="K30" s="13" t="n">
         <x:v>4.99628</x:v>
       </x:c>
-      <x:c r="M3" s="14" t="n">
+      <x:c r="L30" s="14" t="n">
         <x:v>0.1207</x:v>
       </x:c>
-      <x:c r="N3" s="8" t="n">
+      <x:c r="M30" s="8" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="O3" s="8" t="n">
+      <x:c r="N30" s="8" t="n">
         <x:v>7000</x:v>
       </x:c>
-      <x:c r="P3" s="17" t="n">
+      <x:c r="O30" s="17" t="n">
         <x:v>0.84635</x:v>
       </x:c>
-      <x:c r="Q3" s="14" t="n">
+      <x:c r="P30" s="14" t="n">
         <x:v>1.69888</x:v>
       </x:c>
-      <x:c r="R3" s="17" t="n">
+      <x:c r="Q30" s="17" t="n">
         <x:v>5.06443</x:v>
       </x:c>
-      <x:c r="S3" s="14" t="n">
+      <x:c r="R30" s="14" t="n">
         <x:v>0.79788</x:v>
       </x:c>
-      <x:c r="T3" s="17" t="n">
+      <x:c r="S30" s="17" t="n">
         <x:v>0.44289</x:v>
       </x:c>
-      <x:c r="U3" s="14" t="n">
+      <x:c r="T30" s="14" t="n">
         <x:v>1.71308</x:v>
       </x:c>
-      <x:c r="V3" s="10" t="n">
-        <x:f>(AB3/AA3)^2*1000/2*0.000001</x:f>
+      <x:c r="U30" s="10" t="n">
+        <x:f>(AA30/Z30)^2*1000/2*0.000001</x:f>
         <x:v>0.4789679803700033</x:v>
       </x:c>
-      <x:c r="W3" s="19" t="n">
-        <x:f>(V3+L3-3170*0.000001)/V3</x:f>
+      <x:c r="V30" s="19" t="n">
+        <x:f>(U30+K30-3170*0.000001)/U30</x:f>
         <x:v>11.424726087415733</x:v>
       </x:c>
-      <x:c r="X3" s="14" t="n">
-        <x:f>(T3+R3-3170*0.000001)/T3</x:f>
+      <x:c r="W30" s="14" t="n">
+        <x:f>(S30+Q30-3170*0.000001)/S30</x:f>
         <x:v>12.427803743593218</x:v>
       </x:c>
-      <x:c r="Y3" s="14" t="n">
-        <x:f>P3*PI()/4*0.5075*0.5075*0.000001*SQRT(2*1000*T3*1000000)*1000*2</x:f>
+      <x:c r="X30" s="14" t="n">
+        <x:f>O30*PI()/4*0.5075*0.5075*0.000001*SQRT(2*1000*S30*1000000)*1000*2</x:f>
         <x:v>10.190720814760232</x:v>
       </x:c>
-      <x:c r="Z3" s="14" t="n">
-        <x:f>Y3+$Y$2</x:f>
+      <x:c r="Y30" s="14" t="n">
+        <x:f>X30+$X$2</x:f>
         <x:v>10.010720814760232</x:v>
       </x:c>
-      <x:c r="AA3" s="14" t="n">
-        <x:f>Z3/(PI()/4*0.5075*0.5075*SQRT(2*1000*T3))/2</x:f>
+      <x:c r="Z30" s="14" t="n">
+        <x:f>Y30/(PI()/4*0.5075*0.5075*SQRT(2*1000*S30))/2</x:f>
         <x:v>0.8314008121290747</x:v>
       </x:c>
-      <x:c r="AB3" s="14" t="n">
-        <x:f>J3/P3*AA3</x:f>
+      <x:c r="AA30" s="14" t="n">
+        <x:f>I30/O30*Z30</x:f>
         <x:v>25.73230455451408</x:v>
       </x:c>
-      <x:c r="AC3" s="14"/>
-      <x:c r="AD3" s="27" t="str">
+      <x:c r="AB30" s="14"/>
+      <x:c r="AC30" s="27" t="str">
         <x:v>演示处理8000–8019帧；左侧范围保留原始工况记录。</x:v>
       </x:c>
-      <x:c r="AE3" s="2"/>
-      <x:c r="AF3" s="2"/>
-      <x:c r="AG3" s="14" t="n">
+      <x:c r="AD30" s="2"/>
+      <x:c r="AE30" s="2"/>
+      <x:c r="AF30" s="14" t="n">
         <x:v>277</x:v>
       </x:c>
-      <x:c r="AH3" s="14" t="n">
+      <x:c r="AG30" s="14" t="n">
         <x:v>302</x:v>
       </x:c>
-      <x:c r="AI3" s="14" t="n">
+      <x:c r="AH30" s="14" t="n">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="AJ3" s="14" t="n">
+      <x:c r="AI30" s="14" t="n">
         <x:v>250</x:v>
       </x:c>
-      <x:c r="AK3" s="14" t="n">
+      <x:c r="AJ30" s="14" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AL3" s="14" t="n">
+      <x:c r="AK30" s="14" t="n">
         <x:v>1800</x:v>
       </x:c>
-      <x:c r="AM3" s="14" t="n">
+      <x:c r="AL30" s="14" t="n">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="AN3" s="14" t="n">
+      <x:c r="AM30" s="14" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="AO3" s="14" t="n">
+      <x:c r="AN30" s="14" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="AP3" s="14" t="n">
+      <x:c r="AO30" s="14" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AQ3" s="14" t="n">
+      <x:c r="AP30" s="14" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="AR3" s="14" t="n">
+      <x:c r="AQ30" s="14" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="AS3" s="14" t="n">
+      <x:c r="AR30" s="14" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="AT3" s="14" t="n">
+      <x:c r="AS30" s="14" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="AU3" s="14"/>
-      <x:c r="AV3" s="14"/>
-      <x:c r="AW3" s="22"/>
-      <x:c r="AX3" s="14"/>
-      <x:c r="AY3" s="24"/>
-      <x:c r="AZ3" s="22"/>
-      <x:c r="BA3" s="14"/>
-      <x:c r="BB3" s="24"/>
-      <x:c r="BC3" s="22"/>
-      <x:c r="BD3" s="14"/>
-      <x:c r="BE3" s="24"/>
-      <x:c r="BF3" s="22"/>
-      <x:c r="BG3" s="14"/>
-      <x:c r="BH3" s="24"/>
+      <x:c r="AT30" s="14"/>
+      <x:c r="AU30" s="14"/>
+      <x:c r="AV30" s="22"/>
+      <x:c r="AW30" s="14"/>
+      <x:c r="AX30" s="24"/>
+      <x:c r="AY30" s="22"/>
+      <x:c r="AZ30" s="14"/>
+      <x:c r="BA30" s="24"/>
+      <x:c r="BB30" s="22"/>
+      <x:c r="BC30" s="14"/>
+      <x:c r="BD30" s="24"/>
+      <x:c r="BE30" s="22"/>
+      <x:c r="BF30" s="14"/>
+      <x:c r="BG30" s="24"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>